<commit_message>
v1.4 - courts info + map button + UI improvements
</commit_message>
<xml_diff>
--- a/murojaatlar.xlsx
+++ b/murojaatlar.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>№</t>
   </si>
@@ -40,6 +40,27 @@
     <t>Sana</t>
   </si>
   <si>
+    <t>MUR-1777925479252</t>
+  </si>
+  <si>
+    <t>u6</t>
+  </si>
+  <si>
+    <t>ytr</t>
+  </si>
+  <si>
+    <t>yrty</t>
+  </si>
+  <si>
+    <t>Mirzo Ulug‘bek</t>
+  </si>
+  <si>
+    <t>Jinoyat</t>
+  </si>
+  <si>
+    <t>05/05/2026, 01:11:19</t>
+  </si>
+  <si>
     <t>MUR-1777490895731</t>
   </si>
   <si>
@@ -53,9 +74,6 @@
   </si>
   <si>
     <t>Bektemir</t>
-  </si>
-  <si>
-    <t>Jinoyat</t>
   </si>
   <si>
     <t>30/04/2026, 00:28:15</t>
@@ -439,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -505,10 +523,39 @@
         <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>